<commit_message>
cambios en los ws
</commit_message>
<xml_diff>
--- a/RelojUNA-Server/prueba.xlsx
+++ b/RelojUNA-Server/prueba.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="14">
   <si>
     <t>Cantidad de empleados:</t>
   </si>
@@ -44,43 +44,16 @@
     <t>ENTRADA</t>
   </si>
   <si>
+    <t>2026-08-01T08:15</t>
+  </si>
+  <si>
     <t>2026-08-01T17:00</t>
   </si>
   <si>
     <t>SALIDA</t>
   </si>
   <si>
-    <t>2026-08-15</t>
-  </si>
-  <si>
-    <t>2026-08-15T08:00</t>
-  </si>
-  <si>
-    <t>2026-08-15T17:00</t>
-  </si>
-  <si>
-    <t>2026-08-20</t>
-  </si>
-  <si>
-    <t>2026-08-20T18:46:16.651660</t>
-  </si>
-  <si>
-    <t>2026-08-22</t>
-  </si>
-  <si>
-    <t>2026-08-22T13:31:48.279634</t>
-  </si>
-  <si>
-    <t>2026-08-22T14:31:50.417128</t>
-  </si>
-  <si>
-    <t>2026-08-23</t>
-  </si>
-  <si>
-    <t>2026-08-23T09:00</t>
-  </si>
-  <si>
-    <t>2026-08-23T18:00</t>
+    <t>2026-08-01T18:30</t>
   </si>
 </sst>
 </file>
@@ -131,12 +104,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="21.8046875" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="10.13671875" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="24.65234375" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="15.62890625" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="8.69921875" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
@@ -145,7 +118,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="n" s="0">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="2">
@@ -153,7 +126,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="n" s="0">
-        <v>9.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="3">
@@ -161,7 +134,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="n" s="0">
-        <v>27.0</v>
+        <v>19.25</v>
       </c>
     </row>
     <row r="5">
@@ -180,7 +153,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n" s="0">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="B6" t="s" s="0">
         <v>7</v>
@@ -203,105 +176,35 @@
         <v>10</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n" s="0">
-        <v>3.0</v>
+        <v>1.0</v>
       </c>
       <c r="B8" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="D8" t="s" s="0">
         <v>12</v>
-      </c>
-      <c r="C8" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="D8" t="s" s="0">
-        <v>9</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n" s="0">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="B9" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="D9" t="s" s="0">
         <v>12</v>
-      </c>
-      <c r="C9" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="D9" t="s" s="0">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n" s="0">
-        <v>2.0</v>
-      </c>
-      <c r="B10" t="s" s="0">
-        <v>15</v>
-      </c>
-      <c r="C10" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="D10" t="s" s="0">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n" s="0">
-        <v>2.0</v>
-      </c>
-      <c r="B11" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="C11" t="s" s="0">
-        <v>18</v>
-      </c>
-      <c r="D11" t="s" s="0">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n" s="0">
-        <v>2.0</v>
-      </c>
-      <c r="B12" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="C12" t="s" s="0">
-        <v>19</v>
-      </c>
-      <c r="D12" t="s" s="0">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n" s="0">
-        <v>4.0</v>
-      </c>
-      <c r="B13" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="C13" t="s" s="0">
-        <v>21</v>
-      </c>
-      <c r="D13" t="s" s="0">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n" s="0">
-        <v>4.0</v>
-      </c>
-      <c r="B14" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="C14" t="s" s="0">
-        <v>22</v>
-      </c>
-      <c r="D14" t="s" s="0">
-        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>